<commit_message>
EPBDS-17055 Stop teaching deprecated table types in the Reference Guide
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/1-Data-Model/Constants.xlsx
+++ b/DEV/org.openl.rules.demo/src/org.openl.rules.demo.examples/Example-4-Reference-Guide/rules/1-Data-Model/Constants.xlsx
@@ -557,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:I133"/>
+  <dimension ref="B2:I120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
@@ -1192,914 +1192,732 @@
     <row r="59">
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Method Double InvoiceTotal(Double invoiceAmount)</t>
-        </is>
-      </c>
+          <t>Spreadsheet Double InvoiceTotal(Double invoiceAmount)</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="n"/>
     </row>
     <row r="60">
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>Invoice invoice = new Invoice(amount = invoiceAmount);</t>
+      <c r="B60" s="10" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="C60" s="10" t="inlineStr">
+        <is>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>return invoice.amount * (1 + invoice.taxRate);</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="3" t="inlineStr">
+          <t>Invoice</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>= new Invoice(amount = invoiceAmount)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C62" s="8" t="inlineStr">
+        <is>
+          <t>= $Invoice.amount * (1 + $Invoice.taxRate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>Test InvoiceTotal InvoiceTotalTest</t>
         </is>
       </c>
-      <c r="C63" s="5" t="n"/>
-    </row>
-    <row r="64">
-      <c r="B64" s="7" t="inlineStr">
+      <c r="C64" s="5" t="n"/>
+    </row>
+    <row r="65">
+      <c r="B65" s="7" t="inlineStr">
         <is>
           <t>invoiceAmount</t>
         </is>
       </c>
-      <c r="C64" s="7" t="inlineStr">
+      <c r="C65" s="7" t="inlineStr">
         <is>
           <t>_res_</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="B65" s="10" t="inlineStr">
+    <row r="66">
+      <c r="B66" s="10" t="inlineStr">
         <is>
           <t>Amount</t>
         </is>
       </c>
-      <c r="C65" s="10" t="inlineStr">
+      <c r="C66" s="10" t="inlineStr">
         <is>
           <t>Total With Tax</t>
         </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="C66" s="11" t="n">
-        <v>120</v>
       </c>
     </row>
     <row r="67">
       <c r="B67" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="C67" s="11" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="B68" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="C67" s="11" t="n">
+      <c r="C68" s="11" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" s="9" t="inlineStr">
+    <row r="70">
+      <c r="B70" s="9" t="inlineStr">
         <is>
           <t>Other types and empty constants</t>
         </is>
       </c>
     </row>
-    <row r="71" ht="16.5" customHeight="1">
-      <c r="B71" s="2" t="inlineStr">
+    <row r="72" ht="16.5" customHeight="1">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>A constant can have any type that a cell can hold, such as Long, BigDecimal, BigInteger, Character, Float or DoubleRange. A constant without a value is null. A text with only a space needs a formula: = " ".</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="B73" s="3" t="inlineStr">
+    <row r="74">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>Constants MoreConstants</t>
         </is>
       </c>
-      <c r="C73" s="4" t="n"/>
-      <c r="D73" s="5" t="n"/>
-    </row>
-    <row r="74">
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>Long</t>
-        </is>
-      </c>
-      <c r="C74" s="7" t="inlineStr">
-        <is>
-          <t>BIG_COUNT</t>
-        </is>
-      </c>
-      <c r="D74" s="6" t="n">
-        <v>3634</v>
-      </c>
+      <c r="C74" s="4" t="n"/>
+      <c r="D74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>BigDecimal</t>
+          <t>Long</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>EXACT_PRICE</t>
-        </is>
-      </c>
-      <c r="D75" s="6" t="inlineStr">
-        <is>
-          <t>12.35</t>
-        </is>
+          <t>BIG_COUNT</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>3634</v>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>BigInteger</t>
+          <t>BigDecimal</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>HUGE_NUMBER</t>
+          <t>EXACT_PRICE</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>123456789012345678901234567890</t>
+          <t>12.35</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>Short</t>
+          <t>BigInteger</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>SMALL_NUMBER</t>
-        </is>
-      </c>
-      <c r="D77" s="6" t="n">
-        <v>23</v>
+          <t>HUGE_NUMBER</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>123456789012345678901234567890</t>
+        </is>
       </c>
     </row>
     <row r="78">
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>Character</t>
+          <t>Short</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>GRADE_LETTER</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+          <t>SMALL_NUMBER</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="79">
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>Float</t>
+          <t>Character</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>RATIO</t>
-        </is>
-      </c>
-      <c r="D79" s="6" t="n">
-        <v>0.5</v>
+          <t>GRADE_LETTER</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
     </row>
     <row r="80">
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>DoubleRange</t>
+          <t>Float</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>PRICE_BAND</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>500 - 700.01</t>
-        </is>
+          <t>RATIO</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="81">
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>DoubleRange</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>SPACE</t>
-        </is>
-      </c>
-      <c r="D81" s="8" t="inlineStr">
-        <is>
-          <t>= " "</t>
+          <t>PRICE_BAND</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>500 - 700.01</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="B82" s="6" t="inlineStr">
         <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
+        <is>
+          <t>SPACE</t>
+        </is>
+      </c>
+      <c r="D82" s="8" t="inlineStr">
+        <is>
+          <t>= " "</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="6" t="inlineStr">
+        <is>
           <t>Object</t>
         </is>
       </c>
-      <c r="C82" s="7" t="inlineStr">
+      <c r="C83" s="7" t="inlineStr">
         <is>
           <t>NOTHING</t>
         </is>
       </c>
-      <c r="D82" s="6" t="n"/>
-    </row>
-    <row r="84">
-      <c r="B84" s="3" t="inlineStr">
+      <c r="D83" s="6" t="n"/>
+    </row>
+    <row r="85">
+      <c r="B85" s="3" t="inlineStr">
         <is>
           <t>Spreadsheet SpreadsheetResult MoreConstantUsage()</t>
         </is>
       </c>
-      <c r="C84" s="5" t="n"/>
-    </row>
-    <row r="85">
-      <c r="B85" s="10" t="inlineStr">
+      <c r="C85" s="5" t="n"/>
+    </row>
+    <row r="86">
+      <c r="B86" s="10" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="C85" s="10" t="inlineStr">
+      <c r="C86" s="10" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t>NextCount</t>
-        </is>
-      </c>
-      <c r="C86" s="8" t="inlineStr">
-        <is>
-          <t>= BIG_COUNT + 1</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>DoublePrice</t>
+          <t>NextCount</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t>= EXACT_PRICE * 2</t>
+          <t>= BIG_COUNT + 1</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="B88" s="6" t="inlineStr">
         <is>
-          <t>HugeLength</t>
+          <t>DoublePrice</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t>= length(HUGE_NUMBER.toString())</t>
+          <t>= EXACT_PRICE * 2</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Letter</t>
+          <t>HugeLength</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr">
         <is>
-          <t>= GRADE_LETTER</t>
+          <t>= length(HUGE_NUMBER.toString())</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="B90" s="6" t="inlineStr">
         <is>
-          <t>HalfRatio</t>
+          <t>Letter</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t>= RATIO / 2</t>
+          <t>= GRADE_LETTER</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>InBand</t>
+          <t>HalfRatio</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>= contains(PRICE_BAND, 700)</t>
+          <t>= RATIO / 2</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" s="6" t="inlineStr">
         <is>
-          <t>Joined</t>
+          <t>InBand</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t>= DAY_SECONDS + SPACE + NOTHING</t>
+          <t>= contains(PRICE_BAND, 700)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="B93" s="6" t="inlineStr">
         <is>
+          <t>Joined</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr">
+        <is>
+          <t>= DAY_SECONDS + SPACE + NOTHING</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="B94" s="6" t="inlineStr">
+        <is>
           <t>IsEmpty</t>
         </is>
       </c>
-      <c r="C93" s="8" t="inlineStr">
+      <c r="C94" s="8" t="inlineStr">
         <is>
           <t>= NOTHING == null</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="B95" s="3" t="inlineStr">
+    <row r="96">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>Test MoreConstantUsage MoreConstantUsageTest</t>
         </is>
       </c>
-      <c r="C95" s="4" t="n"/>
-      <c r="D95" s="4" t="n"/>
-      <c r="E95" s="4" t="n"/>
-      <c r="F95" s="4" t="n"/>
-      <c r="G95" s="4" t="n"/>
-      <c r="H95" s="4" t="n"/>
-      <c r="I95" s="5" t="n"/>
-    </row>
-    <row r="96">
-      <c r="B96" s="7" t="inlineStr">
+      <c r="C96" s="4" t="n"/>
+      <c r="D96" s="4" t="n"/>
+      <c r="E96" s="4" t="n"/>
+      <c r="F96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n"/>
+      <c r="I96" s="5" t="n"/>
+    </row>
+    <row r="97">
+      <c r="B97" s="7" t="inlineStr">
         <is>
           <t>_res_.$NextCount</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C97" s="7" t="inlineStr">
         <is>
           <t>_res_.$DoublePrice</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D97" s="7" t="inlineStr">
         <is>
           <t>_res_.$HugeLength</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr">
+      <c r="E97" s="7" t="inlineStr">
         <is>
           <t>_res_.$Letter</t>
         </is>
       </c>
-      <c r="F96" s="7" t="inlineStr">
+      <c r="F97" s="7" t="inlineStr">
         <is>
           <t>_res_.$HalfRatio</t>
         </is>
       </c>
-      <c r="G96" s="7" t="inlineStr">
+      <c r="G97" s="7" t="inlineStr">
         <is>
           <t>_res_.$InBand</t>
         </is>
       </c>
-      <c r="H96" s="7" t="inlineStr">
+      <c r="H97" s="7" t="inlineStr">
         <is>
           <t>_res_.$Joined</t>
         </is>
       </c>
-      <c r="I96" s="7" t="inlineStr">
+      <c r="I97" s="7" t="inlineStr">
         <is>
           <t>_res_.$IsEmpty</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="B97" s="10" t="inlineStr">
+    <row r="98">
+      <c r="B98" s="10" t="inlineStr">
         <is>
           <t>Next Count</t>
         </is>
       </c>
-      <c r="C97" s="10" t="inlineStr">
+      <c r="C98" s="10" t="inlineStr">
         <is>
           <t>Double Price</t>
         </is>
       </c>
-      <c r="D97" s="10" t="inlineStr">
+      <c r="D98" s="10" t="inlineStr">
         <is>
           <t>Huge Length</t>
         </is>
       </c>
-      <c r="E97" s="10" t="inlineStr">
+      <c r="E98" s="10" t="inlineStr">
         <is>
           <t>Letter</t>
         </is>
       </c>
-      <c r="F97" s="10" t="inlineStr">
+      <c r="F98" s="10" t="inlineStr">
         <is>
           <t>Half Ratio</t>
         </is>
       </c>
-      <c r="G97" s="10" t="inlineStr">
+      <c r="G98" s="10" t="inlineStr">
         <is>
           <t>In Band</t>
         </is>
       </c>
-      <c r="H97" s="10" t="inlineStr">
+      <c r="H98" s="10" t="inlineStr">
         <is>
           <t>Joined</t>
         </is>
       </c>
-      <c r="I97" s="10" t="inlineStr">
+      <c r="I98" s="10" t="inlineStr">
         <is>
           <t>Is Empty</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="B98" s="11" t="n">
+    <row r="99">
+      <c r="B99" s="11" t="n">
         <v>3635</v>
       </c>
-      <c r="C98" s="11" t="n">
+      <c r="C99" s="11" t="n">
         <v>24.7</v>
       </c>
-      <c r="D98" s="11" t="n">
+      <c r="D99" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="E98" s="11" t="inlineStr">
+      <c r="E99" s="11" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="F98" s="11" t="n">
+      <c r="F99" s="11" t="n">
         <v>0.25</v>
       </c>
-      <c r="G98" s="11" t="inlineStr">
+      <c r="G99" s="11" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="H98" s="11" t="inlineStr">
+      <c r="H99" s="11" t="inlineStr">
         <is>
           <t>86400 null</t>
         </is>
       </c>
-      <c r="I98" s="11" t="inlineStr">
+      <c r="I99" s="11" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="B100" s="9" t="inlineStr">
+    <row r="101">
+      <c r="B101" s="9" t="inlineStr">
         <is>
           <t>Using constants in cells of other tables</t>
         </is>
       </c>
     </row>
-    <row r="102" ht="16.5" customHeight="1">
-      <c r="B102" s="2" t="inlineStr">
-        <is>
-          <t>A constant name in a cell of a Rules table works both as a plain value and as a formula "= NAME". In a ColumnMatch table a constant can be a value, a score or a weight.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="B104" s="3" t="inlineStr">
+    <row r="103" ht="16.5" customHeight="1">
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>A constant name in a cell of a Rules table works both as a plain value and as a formula "= NAME".</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="B105" s="3" t="inlineStr">
         <is>
           <t>Rules String ScoreRating(Integer score)</t>
         </is>
       </c>
-      <c r="C104" s="4" t="n"/>
-      <c r="D104" s="5" t="n"/>
-    </row>
-    <row r="105">
-      <c r="B105" s="7" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="C105" s="5" t="n"/>
-      <c r="D105" s="7" t="inlineStr">
-        <is>
-          <t>RET1</t>
-        </is>
-      </c>
+      <c r="C105" s="4" t="n"/>
+      <c r="D105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>min &lt;= score &amp;&amp; score &lt;= max</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="C106" s="5" t="n"/>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>rating</t>
+          <t>RET1</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" s="7" t="inlineStr">
         <is>
+          <t>min &lt;= score &amp;&amp; score &lt;= max</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="n"/>
+      <c r="D107" s="7" t="inlineStr">
+        <is>
+          <t>rating</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="B108" s="7" t="inlineStr">
+        <is>
           <t>Integer min</t>
         </is>
       </c>
-      <c r="C107" s="7" t="inlineStr">
+      <c r="C108" s="7" t="inlineStr">
         <is>
           <t>Integer max</t>
         </is>
       </c>
-      <c r="D107" s="7" t="inlineStr">
+      <c r="D108" s="7" t="inlineStr">
         <is>
           <t>String rating</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="B108" s="10" t="inlineStr">
+    <row r="109">
+      <c r="B109" s="10" t="inlineStr">
         <is>
           <t>Score From</t>
         </is>
       </c>
-      <c r="C108" s="10" t="inlineStr">
+      <c r="C109" s="10" t="inlineStr">
         <is>
           <t>Score To</t>
         </is>
       </c>
-      <c r="D108" s="10" t="inlineStr">
+      <c r="D109" s="10" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="B109" s="6" t="inlineStr">
+    <row r="110">
+      <c r="B110" s="6" t="inlineStr">
         <is>
           <t>MIN_SCORE</t>
         </is>
       </c>
-      <c r="C109" s="6" t="n">
+      <c r="C110" s="6" t="n">
         <v>579</v>
       </c>
-      <c r="D109" s="11" t="inlineStr">
+      <c r="D110" s="11" t="inlineStr">
         <is>
           <t>Poor</t>
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="B110" s="6" t="n">
+    <row r="111">
+      <c r="B111" s="6" t="n">
         <v>580</v>
       </c>
-      <c r="C110" s="8" t="inlineStr">
+      <c r="C111" s="8" t="inlineStr">
         <is>
           <t>= MAX_SCORE - 1</t>
         </is>
       </c>
-      <c r="D110" s="11" t="inlineStr">
+      <c r="D111" s="11" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="B111" s="6" t="inlineStr">
+    <row r="112">
+      <c r="B112" s="6" t="inlineStr">
         <is>
           <t>MAX_SCORE</t>
         </is>
       </c>
-      <c r="C111" s="6" t="inlineStr">
+      <c r="C112" s="6" t="inlineStr">
         <is>
           <t>MAX_SCORE</t>
         </is>
       </c>
-      <c r="D111" s="11" t="inlineStr">
+      <c r="D112" s="11" t="inlineStr">
         <is>
           <t>Perfect</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="B113" s="3" t="inlineStr">
+    <row r="114">
+      <c r="B114" s="3" t="inlineStr">
         <is>
           <t>Test ScoreRating ScoreRatingTest</t>
         </is>
       </c>
-      <c r="C113" s="5" t="n"/>
-    </row>
-    <row r="114">
-      <c r="B114" s="7" t="inlineStr">
+      <c r="C114" s="5" t="n"/>
+    </row>
+    <row r="115">
+      <c r="B115" s="7" t="inlineStr">
         <is>
           <t>score</t>
         </is>
       </c>
-      <c r="C114" s="7" t="inlineStr">
+      <c r="C115" s="7" t="inlineStr">
         <is>
           <t>_res_</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="B115" s="10" t="inlineStr">
+    <row r="116">
+      <c r="B116" s="10" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="C115" s="10" t="inlineStr">
+      <c r="C116" s="10" t="inlineStr">
         <is>
           <t>Rating</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="B116" s="6" t="n">
-        <v>300</v>
-      </c>
-      <c r="C116" s="11" t="inlineStr">
-        <is>
-          <t>Poor</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="B117" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="C117" s="11" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="6" t="n">
         <v>849</v>
       </c>
-      <c r="C117" s="11" t="inlineStr">
+      <c r="C118" s="11" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="B118" s="6" t="inlineStr">
+    <row r="119">
+      <c r="B119" s="6" t="inlineStr">
         <is>
           <t>MAX_SCORE</t>
         </is>
       </c>
-      <c r="C118" s="11" t="inlineStr">
+      <c r="C119" s="11" t="inlineStr">
         <is>
           <t>Perfect</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="B119" s="6" t="n">
+    <row r="120">
+      <c r="B120" s="6" t="n">
         <v>900</v>
       </c>
-      <c r="C119" s="11" t="n"/>
-    </row>
-    <row r="121">
-      <c r="B121" s="3" t="inlineStr">
-        <is>
-          <t>ColumnMatch &lt;SCORE&gt; Integer CountScore(Long count, Integer score)</t>
-        </is>
-      </c>
-      <c r="C121" s="4" t="n"/>
-      <c r="D121" s="4" t="n"/>
-      <c r="E121" s="4" t="n"/>
-      <c r="F121" s="5" t="n"/>
-    </row>
-    <row r="122">
-      <c r="B122" s="7" t="inlineStr">
-        <is>
-          <t>names</t>
-        </is>
-      </c>
-      <c r="C122" s="7" t="inlineStr">
-        <is>
-          <t>operation</t>
-        </is>
-      </c>
-      <c r="D122" s="7" t="inlineStr">
-        <is>
-          <t>weight</t>
-        </is>
-      </c>
-      <c r="E122" s="7" t="inlineStr">
-        <is>
-          <t>values</t>
-        </is>
-      </c>
-      <c r="F122" s="5" t="n"/>
-    </row>
-    <row r="123">
-      <c r="B123" s="10" t="inlineStr">
-        <is>
-          <t>Attribute</t>
-        </is>
-      </c>
-      <c r="C123" s="10" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="D123" s="10" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="E123" s="10" t="inlineStr">
-        <is>
-          <t>Values</t>
-        </is>
-      </c>
-      <c r="F123" s="5" t="n"/>
-    </row>
-    <row r="124">
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="C124" s="6" t="n"/>
-      <c r="D124" s="6" t="n"/>
-      <c r="E124" s="6" t="inlineStr">
-        <is>
-          <t>RETIREMENT_AGE</t>
-        </is>
-      </c>
-      <c r="F124" s="6" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="C125" s="6" t="inlineStr">
-        <is>
-          <t>match</t>
-        </is>
-      </c>
-      <c r="D125" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E125" s="6" t="inlineStr">
-        <is>
-          <t>BIG_COUNT</t>
-        </is>
-      </c>
-      <c r="F125" s="6" t="inlineStr">
-        <is>
-          <t>0 - 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="C126" s="6" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="D126" s="6" t="inlineStr">
-        <is>
-          <t>RETIREMENT_AGE</t>
-        </is>
-      </c>
-      <c r="E126" s="6" t="inlineStr">
-        <is>
-          <t>MAX_SCORE</t>
-        </is>
-      </c>
-      <c r="F126" s="6" t="inlineStr">
-        <is>
-          <t>MIN_SCORE</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="B128" s="3" t="inlineStr">
-        <is>
-          <t>Test CountScore CountScoreTest</t>
-        </is>
-      </c>
-      <c r="C128" s="4" t="n"/>
-      <c r="D128" s="5" t="n"/>
-    </row>
-    <row r="129">
-      <c r="B129" s="7" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="C129" s="7" t="inlineStr">
-        <is>
-          <t>score</t>
-        </is>
-      </c>
-      <c r="D129" s="7" t="inlineStr">
-        <is>
-          <t>_res_</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="B130" s="10" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C130" s="10" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="D130" s="10" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="B131" s="6" t="n">
-        <v>3634</v>
-      </c>
-      <c r="C131" s="6" t="n">
-        <v>850</v>
-      </c>
-      <c r="D131" s="11" t="n">
-        <v>4355</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="B132" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="C132" s="6" t="n">
-        <v>400</v>
-      </c>
-      <c r="D132" s="11" t="n">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="133">
-      <c r="B133" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="C133" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="D133" s="11" t="n">
-        <v>0</v>
-      </c>
+      <c r="C120" s="11" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="21">
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="B25:I25"/>
+    <mergeCell ref="B59:C59"/>
     <mergeCell ref="B8:D8"/>
-    <mergeCell ref="E122:F122"/>
-    <mergeCell ref="B73:D73"/>
-    <mergeCell ref="B121:F121"/>
-    <mergeCell ref="E123:F123"/>
+    <mergeCell ref="B72:I72"/>
     <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B102:I102"/>
-    <mergeCell ref="B71:I71"/>
-    <mergeCell ref="B105:C105"/>
+    <mergeCell ref="B96:I96"/>
     <mergeCell ref="B19:D19"/>
-    <mergeCell ref="B128:D128"/>
     <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B104:D104"/>
+    <mergeCell ref="B107:C107"/>
+    <mergeCell ref="B74:D74"/>
+    <mergeCell ref="B103:I103"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="B37:I37"/>
-    <mergeCell ref="B84:C84"/>
     <mergeCell ref="B54:D54"/>
+    <mergeCell ref="B64:C64"/>
     <mergeCell ref="B6:I6"/>
-    <mergeCell ref="B95:I95"/>
-    <mergeCell ref="B63:C63"/>
+    <mergeCell ref="B114:C114"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B105:D105"/>
     <mergeCell ref="B106:C106"/>
-    <mergeCell ref="B113:C113"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>